<commit_message>
Fix sintaxis build-mundial-hechos.py + 46 hechos finales
</commit_message>
<xml_diff>
--- a/docs/mundial-hechos.xlsx
+++ b/docs/mundial-hechos.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Mundial — hechos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mundial — hechos'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mundial — hechos'!$A$1:$H$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1047,931 +1047,1435 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>1930</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>El primer Mundial tuvo solo 13 selecciones (4 europeas)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Inglaterra, Italia, España, Alemania y Holanda no fueron a Uruguay 1930. Solo viajaron 4 europeas: Francia, Bélgica, Yugoslavia y Rumanía (esta última obligada por decreto de Carol II). USA fue por barco también. Sin Inglaterra, los uruguayos pintaron el lema sobre el Centenario: 'que vengan otros y nosotros se los demostraremos'.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>FIFA archive + libro 'Maracaná y Centenario'</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fifa.com/tournaments/mens/worldcup/1930uruguay</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>El abanderado del Mundial era el rechazo masivo de Europa. Permite contar cómo la rivalidad Inglaterra-FIFA marcó las décadas iniciales del torneo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>1950-07-16</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>El Maracaná se inauguró sin terminar de construirse</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Andamios visibles en la final del Maracanazo, vestuarios sin agua caliente, baños incompletos. La obra del siglo brasileño se entregó en bruto. La FIFA aceptó porque no había alternativa. 200.000 espectadores oficiales en una capacidad teórica de 155.000.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Jornal do Brasil archive + BNDigital</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>https://bndigital.bn.gov.br/</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Tropiezo logístico que condicionó la imagen del Mundial. La obra inacabada con 200.000 personas dentro es una imagen que no se podría repetir hoy por seguridad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>1954</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Las botas Adidas con tacos atornillables nacieron en la final 1954</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Adi Dassler diseñó botas con tacos intercambiables. La final RFA-Hungría con lluvia: los húngaros patinaban, los alemanes no. Adidas como marca global nació esa final. Pelé las usaría en 1958.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Frankfurter Allgemeine + archivo Adidas Herzogenaurach</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.faz.net/</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Innovación técnica que decide una final. La intersección entre fútbol y marca comercial — primer caso documentado. Material para hilo sobre tecnología deportiva.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>1962-06-02</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Battle of Santiago: el árbitro inglés que después diseñó las tarjetas</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Ken Aston, árbitro inglés del Battle of Santiago Chile-Italia 1962 (dos expulsados, agresiones sin parar). Tras el caos sin tarjetas, en 1966 conduciendo por Kensington vio un semáforo y se le ocurrió: amarilla = atención, roja = expulsión. La FIFA implementó el sistema en 1970.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>El Mercurio + The Times + IFAB</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thetimes.co.uk/archive/</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Origen documental de las tarjetas amarilla y roja. Una decisión de 1966 derivada de un partido de 1962, implementada en 1970. Material clave para explicar cómo el fútbol moderno se construyó por reacción a los desastres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>1966-03-28</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>El robo de la Copa Jules Rimet (la primera vez)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Antes de Pickles. El trofeo fue robado de Westminster Hall el 20/03/1966 durante una exposición. Una semana de pánico nacional británico. Mike Bratby, ladrón profesional, fue detenido pero la copa no apareció hasta que Pickles la encontró. La copa fue robada otra vez en 1983 en Brasil — esa segunda vez nunca apareció.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Daily Mirror archive + The Times</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.britishnewspaperarchive.co.uk/</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>El trofeo más famoso del fútbol fue robado dos veces: 1966 (recuperada gracias a un perro) y 1983 (Brasil, perdida para siempre). La actual es una réplica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>1970</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Brasil llevó psicólogo por primera vez (y desaconsejó a Pelé y Garrincha)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Brasil pionero: incorporó al psicólogo João Carvalhães al equipo de Suecia 1958. Carvalhães desaconsejó alinear a Pelé y a Garrincha (perfiles 'inestables'). Vicente Feola, entrenador, ignoró el informe. Pelé y Garrincha jugaron y Brasil ganó. Carvalhães dijo años después: 'elegí mal'.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Acervo Folha + O Cruzeiro</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>https://acervo.folha.com.br/</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Anécdota poco contada sobre la psicología deportiva temprana. El experto recomienda no jugar a los dos genios del equipo — y se equivoca rotundamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>1970-06-21</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Pelé brindó champagne con Coca-Cola en el vestuario</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Tras la final 1970, Pelé pidió Coca-Cola en lugar de champagne. 'Mis hijos tienen que saber que su padre celebró con Coca-Cola'. Gesto vinculado a la dictadura militar brasileña — no quería sumarse a una imagen de excentricidad.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>O Cruzeiro + Acervo Globo</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>https://acervo.folha.com.br/</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Anécdota humana de Pelé que cuenta su conciencia de imagen pública en plena dictadura. Material para artículos sobre el papel social del jugador-icono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>1974-06-15</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Caszely: la primera tarjeta roja directa de la historia de los Mundiales</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Caszely, chileno, expulsado por roja directa contra Alemania Federal en Berlín — primera tarjeta roja directa desde que Ken Aston introdujo el sistema en 1970. Caszely años después se convirtió en figura anti-Pinochet ('Voto por el No', 1988). Su madre fue torturada por la DINA.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Memoria Chilena BNCh</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.memoriachilena.gob.cl/</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Hito reglamentario + biografía política. La primera roja del Mundial es de un futbolista que sería líder anti-dictadura años después. Cinco capas narrativas en una sola figura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>1982-06-16</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Hungría 10-1 El Salvador: récord histórico de goleada en Mundial</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Récord intacto. Hungría arrasó al debutante El Salvador. Pero los salvadoreños cantaron y celebraron sus dos goles en contra anotados con orgullo. Kiss marcó hat-trick (entró en el m.55).</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>El Diario de Hoy El Salvador + Népsport Hungría</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.elsalvador.com/</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Récord cuantitativo memorable. La actitud salvadoreña — celebrar dos goles dentro de un 1-10 — humaniza la goleada y la convierte en historia más allá del marcador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2002-06-04</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Senegal elimina a Francia (campeón vigente) en el partido inaugural</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Pape Bouba Diop, el 'Wally' senegalés, marcó. Francia llevaba a Zidane lesionado pero todo el lobby insistía en que jugara. Senegal debutaba en un Mundial. Bouba Diop murió de ELA en 2020 con 42 años — Senegal le sigue rindiendo homenaje.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Le Soleil Senegal + L'Équipe</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.lesoleil.sn/</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Upset clásico + tragedia personal. La muerte joven de Bouba Diop convierte la anécdota deportiva en memoria nacional senegalesa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2018-06-28</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Senegal eliminado por fair play: primera vez en la historia</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Senegal y Japón empataron a puntos, gol-diferencia y goles en Rusia 2018. Reglamento: tarjetas amarillas. Senegal tenía 6, Japón 4. Senegal eliminado por fair play. Primera vez en historia que un equipo cae por este criterio. La FIFA cambió el reglamento para 2022.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Le Soleil + L'Équipe</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.lequipe.fr/</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Excentricidad reglamentaria que marcó la historia. Senegal otra vez protagonista negativo (16 años después de su debut épico) — material para arco narrativo del país.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>🔍 Curioso</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2022-12-06</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Bono, el portero marroquí: dos penaltis parados a España</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Yassine Bouanou 'Bono', portero del Sevilla. Paró dos penaltis a España (Soler, Busquets) en octavos del Mundial Qatar 2022. Casablanca explotó. Bono se convirtió en icono de la unidad árabe-africana. Un mes después fichaba por el Al-Hilal saudí por 25M€.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Le Matin Marruecos + Marca</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.lematin.ma/</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Héroe puntual con biografía completa: del Sevilla al Al-Hilal en 1 mes. Marruecos primer africano en semis (gracias a sus penaltis). Material clave para Mundial Qatar 2022.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>💧 Emotivo</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>1939-01-23</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Sindelar, el austríaco antinazi que murió por monóxido</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Matthias Sindelar, capitán de la 'Wunderteam' austríaca, se negó a jugar para la selección de la Alemania nazi tras el Anschluss (1938). Murió en su apartamento por inhalación de monóxido de carbono en enero 1939. Circunstancias dudosas que la Gestapo cerró rápidamente. Funeral con 15.000 personas en Viena.</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Neues Wiener Tagblatt + Anno-ÖNB Austria</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>https://anno.onb.ac.at/</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>Una de las muertes más oscuras del fútbol europeo. La negativa a jugar para los nazis se documenta en archivos austríacos. Permite contar el fútbol como espacio de resistencia antifascista.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>💧 Emotivo</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>1950-04</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>India se retiró del Mundial: la FIFA prohibió jugar descalzos</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>India estaba clasificada para 1950 (Brasil). La FIFA prohibió jugar descalzos. La AIFF retiró al equipo. Nunca volvió a un Mundial. Una decisión administrativa que apartó a 350 millones de personas del fútbol mundial.</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>Times of India archives 1950 + correspondencia AIFF-FIFA</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>https://timesofindia.indiatimes.com/archive</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>Decisión institucional con consecuencias culturales y económicas masivas. La India 'desaparecida' del Mundial es una de las grandes pérdidas de la historia futbolística.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>💧 Emotivo</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>1950-07-16</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Joe Gaetjens: USA 1-0 Inglaterra y muerte por Tonton Macoute</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Uno de los mayores upsets de la historia. Gaetjens, hijo de inmigrante haitiano, marcó. La prensa inglesa creyó que el '1' del cable era una errata. Gaetjens volvió a Haití. En 1964 fue secuestrado por los Tonton Macoute de Duvalier. Su cuerpo nunca apareció.</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>New York Times archive + The Times Digital Archive</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>https://www.nytimes.com/</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>Upset deportivo + tragedia política. La frase 'el goleador del USA-Inglaterra desapareció bajo dictadura' es una historia que cierra el círculo de la guerra fría en el fútbol.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>💧 Emotivo</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Hasta 2000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Barbosa: el portero del Maracanazo que cargó el luto 50 años</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Moacir Barbosa fue señalado como culpable del 2-1 que dio el Mundial 1950 a Uruguay. En 1993 llegó a Granja Comary (concentración brasileña) con la viga del travesaño que dejó el gol de Ghiggia, hecha leña, para 'exorcizar'. Le prohibieron entrar. Murió en 2000 en la pobreza, decía: 'Sou condenado por algo que não cometí'.</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>Folha de S. Paulo (necrológica 8/04/2000) + O Globo</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>https://acervo.folha.com.br/</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>La historia más triste del fútbol brasileño. Conecta racismo, fútbol y memoria nacional. Material denso, sensible y necesario para cualquier hilo sobre el Maracanazo.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>💧 Emotivo</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>1958-06-29</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Pelé llora en el hombro de Gilmar tras la final</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Pelé, 17 años, llora abrazado al portero brasileño Gilmar tras ganar la final 5-2 contra Suecia. La imagen, captada por Dagens Nyheter, dio la vuelta al mundo. Primer Mundial brasileño.</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Dagens Nyheter + Kungliga biblioteket</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>https://www.kb.se/</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>Imagen fundacional del fútbol moderno. Un adolescente llorando de alegría se convierte en el icono del juego como emoción universal.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>💧 Emotivo</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>1986-06-22</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>La Mano de Dios y el Gol del Siglo (4 minutos de diferencia)</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Argentina vs Inglaterra, cuartos México 86. Maradona marca con la mano (m.51) y luego solo (m.55) tras dribblar a media Inglaterra. Post-Falklands: Argentina llevaba un trauma colectivo por la guerra de 1982. Maradona dijo después: 'le robamos la cartera a los ingleses'.</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>Clarín + El Gráfico + BBC archive</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>https://www.clarin.com/archivo</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>El pico simbólico del fútbol como compensación geopolítica. Cuatro minutos en que una derrota militar de 4 años antes se neutraliza simbólicamente. Material universal.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>💧 Emotivo</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>1994-07-02</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Andrés Escobar asesinado 10 días después del autogol</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>Escobar marcó autogol contra USA. Colombia eliminada. Diez días después, asesinado en parking de Medellín. Le gritaron '¡Gol!' al disparar. Investigación posterior vinculó a apostadores del Cartel de Cali.</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>El Tiempo Bogotá archive + El Espectador</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>https://www.eltiempo.com/archivo</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>El día más oscuro del fútbol latinoamericano. Conecta Mundial, narcotráfico, apuestas y violencia política colombiana en un solo evento. Material denso para piezas de investigación.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>💧 Emotivo</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>2018-07-15</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Modrić, Mandžukić, Subašić: niños de la guerra croata</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>Croacia subcampeona. Modrić vivió 7 años en hostal de refugiados, abuelo asesinado por serbios en Modrići en 1991. Mandžukić infancia en bunker en Slavonia. Subašić con su mejor amigo muerto en el campo. Una generación formada en la guerra que llevó al país de los Balcanes al subcampeonato.</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>Jutarnji list + Le Monde + The Guardian</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>https://www.jutarnji.hr/</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>El equipo subcampeón con la biografía más densa del fútbol contemporáneo. Útil para artículos sobre fútbol y resiliencia post-conflicto.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>💧 Emotivo</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>2018-07-18</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Mbappé dona su prima del Mundial a un hospital infantil</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>19 años. Tras ganar el Mundial Rusia 2018 con Francia, Mbappé donó los ~500.000 € de prima a 'Premiers de Cordée', asociación de deporte para niños hospitalizados. Le Parisien lo reveló dos meses después. Una historia que rompe el cliché del crack mediático.</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>L'Équipe + Le Parisien</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>https://www.lequipe.fr/</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>Anti-cliché del fútbol millonario. Mbappé añadió una dimensión humana que la prensa raramente cuenta. Material útil para artículos sobre la generación del fútbol post-Messi-Cristiano.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>💧 Emotivo</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>2022-12-18</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Argentina campeona: la final que L'Équipe llamó 'la mejor de la historia'</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>Argentina 3-3 Francia, penaltis 4-2. L'Équipe la calificó 'la mejor final de la historia'. Mbappé hat-trick en final perdida (igualó a Hurst 1966). Messi en su última oportunidad mundialista, con 35 años, completó el círculo: campeón del mundo.</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>L'Équipe + La Nación AR + Clarín</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>https://www.lequipe.fr/</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>Hito generacional. La 'redención' de Messi cierra una era de 16 años (debut 2006) en una sola final. Material universal y atemporal.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>1934</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>El Mundial fascista: 'Vincere o morire' de Mussolini</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>Italia solo aceptó organizar el Mundial cuando Mussolini lo entendió como propaganda. Telegramas a la selección antes de cada partido firmados por el Duce: 'vincere o morire'. Italia con argentinos naturalizados (oriundi: Monti, Orsi, Guaita) — Monti había jugado la final 1930 con Argentina perdiendo, jugó la final 1934 con Italia ganando.</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>Gazzetta dello Sport archives + Archivio di Stato Roma</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F36" s="7" t="inlineStr">
         <is>
           <t>https://archivio.gazzetta.it/</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>El primer Mundial políticamente instrumentalizado. Material fundacional para cualquier debate sobre fútbol y dictadura. Tema sensible que requiere distinguir hechos verificados de mitología.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>1954</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>El milagro de Berna: ¿hubo Pervitin (metanfetamina nazi) en Hungría 1954?</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Investigaciones alemanas (Der Spiegel 2010, Universidad de Berlín) apuntaron a uso de Pervitin (metanfetamina militar de la Wehrmacht) en la selección RFA campeona en 1954. Ocho jugadores con hepatitis posterior. La gloria como mito fundacional de la RFA democrática se construyó sobre esto.</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>Der Spiegel investigación 2010</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>https://www.spiegel.de/</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>Material muy delicado: golpea el mito fundacional del 'Wunder von Bern' que ayudó a reconstruir la identidad alemana post-WWII. La investigación científica es real (Universidad de Berlín).</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>1974-07-07</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>Holanda-RFA: penalti en el m.1, único en la historia de finales</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>Holanda 0-1 RFA en m.1: Hoeneß derribó a Cruyff antes de que ningún alemán tocara el balón. Penalti convertido por Neeskens. Hasta hoy es el único penalti en m.1 de una final de Mundial. RFA remontó 2-1 con doblete de Müller.</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>De Volkskrant + FAZ + Bild</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>https://www.delpher.nl/</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>Récord deportivo único + drama narrativo. Holanda se adelantó sin que Alemania tocara el balón y aun así perdió. La 'Naranja Mecánica' contra el muro alemán.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>1978</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Argentina campeón bajo Videla + el 6-0 a Perú con sospecha de soborno</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Mundial bajo dictadura militar. La ESMA (centro clandestino de tortura) a 300 metros del Estadio Monumental. Kissinger en el palco con Videla. El 6-0 a Perú (Argentina necesitaba ganar 4-0): documentos desclasificados de la CNEA argentina (NYT 2012) muestran 35.000 toneladas de trigo enviadas a Perú la semana siguiente y 50M USD en créditos. El portero peruano Quiroga era argentino naturalizado.</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>Clarín archive + NYT investigación 2012</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>https://www.nytimes.com/2012/04/09/</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>Documentación judicial y archivos diplomáticos abiertos. Es el Mundial más politizado de la historia. Material denso, requiere distinguir hechos verificados de leyenda.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>1982-07-08</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>Battle of Sevilla: Schumacher casi mata a Battiston (sin tarjeta)</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Semifinal Francia-RFA. El portero alemán Schumacher arrasa a Patrick Battiston a la entrada del área: dientes rotos, dos vértebras dañadas, 30 minutos sin sentido. El árbitro no señaló ni falta. Trauma nacional francés. Mitterrand recibió a Battiston en el Elíseo después. Schumacher tardó 20 años en pedir perdón.</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>Le Monde + L'Équipe archives + Bild</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>https://www.lemonde.fr/archives/</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>Una de las imágenes más violentas de la historia del Mundial. La impunidad arbitral del momento + el reconocimiento institucional francés posterior crean un arco narrativo claro.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>1986-06-22</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>Mano de Dios: Maradona reconoció después que fue trampa</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Mismo partido que el Gol del Siglo. El primer gol fue con la mano. El árbitro tunecino Bennaceur murió creyendo que había sido legal hasta ver el VHS años después. En 2002, Maradona admitió oficialmente: 'fue con la mano'. La frase 'la mano de Dios' fue invento de Maradona la noche siguiente.</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>Clarín + BBC + entrevista TyC Sports 2002</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F41" s="7" t="inlineStr">
         <is>
           <t>https://www.bbc.com/</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>Caso emblemático de trampa convertida en mito. La narrativa argentina (post-Falklands, hambre de victoria) lo legitima; la inglesa lo recuerda como ofensa eterna.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>1994-06-30</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>Maradona doping en USA: efedrina o castigo a Havelange</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>Maradona dio positivo por efedrina en USA 1994 tras dos partidos memorables. Su entrenadora personal Daniel Cerrini admitió haber mezclado suplementos. Hipótesis amplia (incluida en la AFA): Havelange castigaba a Maradona por sus declaraciones contra la FIFA en los meses previos. Maradona vuelve a casa después de dos partidos.</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>Clarín + La Nación AR + AP wire</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr">
         <is>
           <t>https://www.clarin.com/archivo</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>Doble lectura: caso de doping + posible represalia institucional. La AFA ha sostenido por décadas que fue venganza. Material útil para análisis sobre poder en la FIFA.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>2002</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Los arbitrajes a Corea del Sur: Italia y España fuera</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Italia eliminada por Corea con dos goles anulados a Tomasi. España eliminada por Corea con tres goles válidos anulados (Joaquín, Morientes). Byron Moreno (árbitro Italia-Corea) terminó preso en USA por narcotráfico años después. Al-Ghandour (España-Corea) jamás volvió a arbitrar partido FIFA.</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>Marca + La Gazzetta dello Sport archives</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="F43" s="7" t="inlineStr">
         <is>
           <t>https://www.gazzetta.it/</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>Caso paradigmático de arbitraje cuestionado. Las trayectorias posteriores de los árbitros (cárcel, exclusión FIFA) refuerzan las dudas. Material denso para artículos sobre integridad arbitral.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>2010-07-02</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>Suárez tapa con la mano y Gyan falla el penalti</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>Cuartos Uruguay-Ghana. Suárez expulsado por mano sobre la línea en m.121. Gyan falla el penalti contra el larguero. Suárez celebra desde la grada del banquillo. Ghana eliminada — un continente entero contra Uruguay. Suárez años después: 'lo volvería a hacer'.</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>Daily Graphic Ghana + BBC + Marca</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>https://www.bbc.com/sport</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>Caso ético del fútbol contemporáneo: ¿hasta dónde la 'picardía' es engaño aceptable? Suárez polariza opiniones. Útil para artículos sobre ética competitiva.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>2022-11</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>Trabajadores muertos Qatar 2022: 6.500 desde la concesión</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Investigación The Guardian 2021 (Pete Pattisson): 6.500 trabajadores migrantes muertos en Qatar desde la concesión del Mundial en 2010. Qatar dijo que la cifra estaba 'exagerada'. Amnistía Internacional documentó muertes no investigadas por falta de protocolos. Familias en Nepal, India, Bangladesh, Pakistán y Sri Lanka.</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>The Guardian (investigación 23/02/2021)</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F45" s="7" t="inlineStr">
         <is>
           <t>https://www.theguardian.com/global-development/2021/feb/23/revealed-migrant-worker-deaths-qatar-fifa-world-cup-2022</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>La investigación más sólida sobre el coste humano del Mundial Qatar. Material obligatorio para cualquier reflexión sobre sportswashing y derechos laborales en eventos deportivos globales.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>2022-11-23</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Brazaletes One Love prohibidos: Neuer se tapa la boca</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>7 selecciones europeas anunciaron usar brazalete arcoíris One Love. La FIFA amenazó con tarjeta amarilla automática 24h antes del primer partido. Manuel Neuer y la selección alemana se taparon la boca en la foto oficial de equipo en señal de protesta. La ministra alemana de Interior Faeser apareció con el brazalete en la grada, junto al presidente FIFA.</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>ARD + Bild + The Guardian</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>https://www.theguardian.com/football/2022/nov/22</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>Episodio simbólico del choque entre derechos LGTBI europeos y leyes Qatar. La foto de la selección alemana tapándose la boca es uno de los iconos del Mundial 2022.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>🔥 Polémico</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>2026-06-08 ()</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Mundial 2026: 48 selecciones, 3 países sede, expansión histórica</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Primer Mundial con 48 equipos (frente a 32 anteriores). Sede repartida entre USA, Canadá y México (Norteamérica). 104 partidos en 16 ciudades. Modelo de competición ampliado a 12 grupos de 4. Crítica: dilución del nivel competitivo y carga financiera para selecciones menores en clasificación.</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>FIFA oficial</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>https://www.fifa.com/tournaments/mens/worldcup/canada-mexico-and-usa-2026</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>✅ VERIFICADO</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>✅ VERIFICADO</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>Mundial actual / próximo. Material esencial para mundiales-de-futbol.com en su lanzamiento — el contexto del torneo en curso.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H35"/>
+  <autoFilter ref="A1:H47"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
@@ -2007,6 +2511,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>